<commit_message>
Note the number of samples in each data set used to train the model to check the fairness of the comparison between different subsets (mfc type, resistance, year)
</commit_message>
<xml_diff>
--- a/model_performance_.xlsx
+++ b/model_performance_.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uob-my.sharepoint.com/personal/hp12384_bristol_ac_uk/Documents/Projects/APEX/APEX_WP2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_5BDFEDE98B0CD465CF41CF74302E021479DD994B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{521B4042-6A16-9644-9DE2-632F7A332882}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_5BDFEDE98B0CD465CF41CF74302E021479DD994B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D63637DE-F4C3-1546-934C-E0B010F312BC}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ridge" sheetId="1" r:id="rId1"/>
@@ -208,10 +208,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -728,8 +724,11 @@
   <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="36.33203125" customWidth="1"/>
     <col min="3" max="3" width="31.1640625" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
+    <col min="10" max="10" width="25" customWidth="1"/>
+    <col min="11" max="11" width="31.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">

</xml_diff>